<commit_message>
Add training section on attributor combiner
</commit_message>
<xml_diff>
--- a/training/training_datasets.xlsx
+++ b/training/training_datasets.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849E7E48-4774-4AAD-80BF-26DC55362E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126B32B8-1FBE-4DD0-9DF7-7454DEF8B0F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10440" yWindow="-13080" windowWidth="17280" windowHeight="8880" xr2:uid="{6AB19A42-3001-43E5-B0C9-18958D7707B1}"/>
+    <workbookView xWindow="6210" yWindow="-12435" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{6AB19A42-3001-43E5-B0C9-18958D7707B1}"/>
   </bookViews>
   <sheets>
     <sheet name="msr_creator" sheetId="1" r:id="rId1"/>
+    <sheet name="attributor_combiner" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>file_name_regions</t>
   </si>
@@ -50,15 +51,9 @@
     <t>file_name_region_boundaries</t>
   </si>
   <si>
-    <t>AllCountryBoundaries_GAUL</t>
-  </si>
-  <si>
     <t>file_name_population_density</t>
   </si>
   <si>
-    <t>lspop2015</t>
-  </si>
-  <si>
     <t>file_name_urban_area_load_centers</t>
   </si>
   <si>
@@ -68,69 +63,36 @@
     <t>file_name_land_cover</t>
   </si>
   <si>
-    <t>GLOBCOVER_L4_200901_200912_V2.3</t>
-  </si>
-  <si>
     <t>file_name_elevation</t>
   </si>
   <si>
-    <t>srtm30_e_w_merged</t>
-  </si>
-  <si>
     <t>file_name_climate_classes</t>
   </si>
   <si>
-    <t>koppen_geiger_0p00833333</t>
-  </si>
-  <si>
     <t>file_name_protected_areas</t>
   </si>
   <si>
-    <t>WDPA_Mar2026</t>
-  </si>
-  <si>
     <t>file_name_water_bodies</t>
   </si>
   <si>
-    <t>HydroLAKES_polys_v10</t>
-  </si>
-  <si>
     <t>file_name_roads</t>
   </si>
   <si>
-    <t>Roads_GRIPGlobal</t>
-  </si>
-  <si>
     <t>file_name_substations</t>
   </si>
   <si>
-    <t>OSM_Substations</t>
-  </si>
-  <si>
     <t>file_name_power_grid</t>
   </si>
   <si>
-    <t>gridfinder_allTDgrid</t>
-  </si>
-  <si>
     <t>file_name_transmission_grid</t>
   </si>
   <si>
-    <t>gridfinder_T</t>
-  </si>
-  <si>
     <t>file_name_continent_distance_surface_tgrid</t>
   </si>
   <si>
-    <t>ContinentalDistanceSurface_gridfinder_T</t>
-  </si>
-  <si>
     <t>file_name_distribution_grid</t>
   </si>
   <si>
-    <t>gridfinder_D</t>
-  </si>
-  <si>
     <t>file_name_buffer_distance</t>
   </si>
   <si>
@@ -140,21 +102,12 @@
     <t>file_name_ghi_map</t>
   </si>
   <si>
-    <t>GHI_2026</t>
-  </si>
-  <si>
     <t>file_name_wind_speed_map</t>
   </si>
   <si>
-    <t>ECU_wind-speed_100m</t>
-  </si>
-  <si>
     <t>file_name_dni_map</t>
   </si>
   <si>
-    <t>DNI</t>
-  </si>
-  <si>
     <t>file_name_climate_class_legend</t>
   </si>
   <si>
@@ -165,14 +118,102 @@
   </si>
   <si>
     <t>land_cover_legend</t>
+  </si>
+  <si>
+    <t>ECU_boundaries</t>
+  </si>
+  <si>
+    <t>ECU_lspop</t>
+  </si>
+  <si>
+    <t>ECU_GLOBCOVER</t>
+  </si>
+  <si>
+    <t>ECU_SRTM</t>
+  </si>
+  <si>
+    <t>ECU_koppen_geiger</t>
+  </si>
+  <si>
+    <t>ECU_WDPA</t>
+  </si>
+  <si>
+    <t>ECU_HydroLAKES</t>
+  </si>
+  <si>
+    <t>ECU_GRIP</t>
+  </si>
+  <si>
+    <t>ECU_gridfinder_allTDgrid</t>
+  </si>
+  <si>
+    <t>ECU_gridfinder_T</t>
+  </si>
+  <si>
+    <t>ECU_gridfinder_D</t>
+  </si>
+  <si>
+    <t>ECU_GHI</t>
+  </si>
+  <si>
+    <t>ECU_wind_speed_100m</t>
+  </si>
+  <si>
+    <t>ECU_OSM_S</t>
+  </si>
+  <si>
+    <t>region_names.csv</t>
+  </si>
+  <si>
+    <t>file_name_resource_raster</t>
+  </si>
+  <si>
+    <t>file_name_cost_assumptions</t>
+  </si>
+  <si>
+    <t>cost_assumptions.csv</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">or </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ECU_GHI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  for solar PV</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -538,6 +579,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{539C2FE2-F2FD-4E88-92E0-49AB48D59D00}">
   <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="39.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -552,159 +596,193 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{222F6492-4F89-4075-98FA-27EB1CC5CF58}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>